<commit_message>
feat: add Jedox Partners and Offer Mail email templates and update test mail data.
</commit_message>
<xml_diff>
--- a/Test Mail.xlsx
+++ b/Test Mail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,11 +449,11 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46056</v>
+        <v>46077</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sent at 2026-02-03 17:09:30</t>
+          <t>Sent at 2026-02-24 10:25:18</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,18 +465,58 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mashal@finlytyx.com</t>
+          <t>swathy@finlytyx.com</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46056</v>
+        <v>46077</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sent at 2026-02-03 17:09:32</t>
+          <t>Sent at 2026-02-24 10:30:28</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
+        <is>
+          <t>Offer Mail.msg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>shanitha@finlytyx.com</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46077</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sent at 2026-02-24 10:25:22</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Jedox Partners.msg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>shameem@finlytyx.com</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46077</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sent at 2026-02-24 10:25:24</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Power BI.msg</t>
         </is>

</xml_diff>

<commit_message>
feat: Implement email personalization for templates and improve date column parsing in the automation script.
</commit_message>
<xml_diff>
--- a/Test Mail.xlsx
+++ b/Test Mail.xlsx
@@ -417,26 +417,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Mail ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Templates</t>
         </is>
@@ -445,18 +450,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Adil Cholas</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>adil@finlytyx.com</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>46077</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Sent at 2026-02-24 10:25:18</t>
-        </is>
+      <c r="C2" s="1" t="n">
+        <v>46080</v>
       </c>
       <c r="D2" t="inlineStr">
+        <is>
+          <t>Sent at 2026-02-27 12:37:51</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Customer Mail New.msg</t>
         </is>
@@ -465,18 +475,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Swathy</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>swathy@finlytyx.com</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
-        <v>46077</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Sent at 2026-02-24 10:30:28</t>
-        </is>
+      <c r="C3" s="1" t="n">
+        <v>46080</v>
       </c>
       <c r="D3" t="inlineStr">
+        <is>
+          <t>Sent at 2026-02-27 12:37:53</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Offer Mail.msg</t>
         </is>
@@ -485,18 +500,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Shanitha</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>shanitha@finlytyx.com</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>46077</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sent at 2026-02-24 10:25:22</t>
-        </is>
+      <c r="C4" s="1" t="n">
+        <v>46080</v>
       </c>
       <c r="D4" t="inlineStr">
+        <is>
+          <t>Sent at 2026-02-27 12:37:55</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Jedox Partners.msg</t>
         </is>
@@ -505,18 +525,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Shameem</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>shameem@finlytyx.com</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>46077</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Sent at 2026-02-24 10:25:24</t>
-        </is>
+      <c r="C5" s="1" t="n">
+        <v>46080</v>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>Sent at 2026-02-27 12:37:58</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Power BI.msg</t>
         </is>

</xml_diff>

<commit_message>
feat(frontend): add multi-page dashboard with backend integration
- Replace default React app with multi-page dashboard layout
- Add pages for templates, recipients, history, and settings
- Implement backend API integration using FastAPI with endpoints for stats, logs, templates, and recipients
- Add file upload functionality for Excel campaigns
- Include real-time automation status control and log viewing
- Update frontend dependencies to include axios and react-router-dom
</commit_message>
<xml_diff>
--- a/Test Mail.xlsx
+++ b/Test Mail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,100 +450,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Adil Cholas</t>
+          <t>Gokul</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>adil@finlytyx.com</t>
+          <t>gokuldaskannadas@gmail.com</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>46080</v>
+        <v>46125</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sent at 2026-02-27 12:37:51</t>
+          <t>Sent at 2026-04-13 23:48:22</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>Customer Mail New.msg</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Swathy</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>swathy@finlytyx.com</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>46080</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Sent at 2026-02-27 12:37:53</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Offer Mail.msg</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Shanitha</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>shanitha@finlytyx.com</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>46080</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Sent at 2026-02-27 12:37:55</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Jedox Partners.msg</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Shameem</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>shameem@finlytyx.com</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>46080</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Sent at 2026-02-27 12:37:58</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Power BI.msg</t>
         </is>
       </c>
     </row>

</xml_diff>